<commit_message>
BRD-13 Data Migration document set v1.0: sign-off form layout, short sheet names
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01W3DAuLtsQmip7EuxjJCCtN
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Migration/BIBS_Migration_BRD-13_Data_Requirements_Workbook_v1.0.xlsx
+++ b/docs/deliverables/out/Migration/BIBS_Migration_BRD-13_Data_Requirements_Workbook_v1.0.xlsx
@@ -11,33 +11,33 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Object Register" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="File Contract" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R01 Lists of values and MIS" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R02 Branches and invoicing" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R03 Sales organisation units" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R01 LOV and MIS values" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R02 Branches" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R03 Sales organisation" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R04 Insurers" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R04B Insurer branches" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R05 Product lines, cover types," sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R06 Packages active versions" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R07 Commission rates by insurer" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R08 Chart of accounts mapping" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R05 Products and risk codes" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R06 Packages" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R07 Commission rates" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R08 GL account map" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R09 Payees" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R11 Receipt series in use" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R11 Receipt series" sheetId="15" state="visible" r:id="rId15"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="C01 Client master" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="C02 Client addresses and" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="C03 Client payout accounts" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P01 In-force policy headers" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P01S Policy insurer shares" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P03 RMEL cohorts already" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F01 Invoices header" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F01S Invoices insurer shares" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F01C Invoices components and" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F02 Unapplied premium payments" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="C02 Client addresses" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="C03 Payout accounts" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P01 Policy headers" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P01S Policy shares" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P03 RMEL cohorts" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F01 Invoice header" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F01S Invoice shares" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F01C Invoice components" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F02 UPP" sheetId="25" state="visible" r:id="rId25"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F03 Open collection state" sheetId="26" state="visible" r:id="rId26"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F04 Remittance in flight" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F06 PDCs, check pick-ups and" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="G01 GL opening trial balance" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="H01 Archive records closed" sheetId="30" state="visible" r:id="rId30"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="H02 Archive documents index" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F06 PDCs pick-ups refunds" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="G01 GL trial balance" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="H01 Archive records" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="H02 Archive documents" sheetId="31" state="visible" r:id="rId31"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control File" sheetId="32" state="visible" r:id="rId32"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control Example" sheetId="33" state="visible" r:id="rId33"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control Totals" sheetId="34" state="visible" r:id="rId34"/>
@@ -55,60 +55,60 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Object Register'!$4:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'File Contract'!$A$4:$B$18</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'File Contract'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'R01 Lists of values and MIS'!$A$4:$L$12</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="4">'R01 Lists of values and MIS'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'R02 Branches and invoicing'!$A$4:$L$9</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="5">'R02 Branches and invoicing'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'R03 Sales organisation units'!$A$4:$L$15</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="6">'R03 Sales organisation units'!$4:$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'R01 LOV and MIS values'!$A$4:$L$12</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="4">'R01 LOV and MIS values'!$4:$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'R02 Branches'!$A$4:$L$9</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="5">'R02 Branches'!$4:$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'R03 Sales organisation'!$A$4:$L$15</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="6">'R03 Sales organisation'!$4:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'R04 Insurers'!$A$4:$L$14</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="7">'R04 Insurers'!$4:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'R04B Insurer branches'!$A$4:$L$11</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="8">'R04B Insurer branches'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'R05 Product lines, cover types,'!$A$4:$L$13</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="9">'R05 Product lines, cover types,'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'R06 Packages active versions'!$A$4:$L$14</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="10">'R06 Packages active versions'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'R07 Commission rates by insurer'!$A$4:$L$9</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="11">'R07 Commission rates by insurer'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'R08 Chart of accounts mapping'!$A$4:$L$12</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="12">'R08 Chart of accounts mapping'!$4:$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'R05 Products and risk codes'!$A$4:$L$13</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="9">'R05 Products and risk codes'!$4:$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'R06 Packages'!$A$4:$L$14</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="10">'R06 Packages'!$4:$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'R07 Commission rates'!$A$4:$L$9</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="11">'R07 Commission rates'!$4:$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'R08 GL account map'!$A$4:$L$12</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="12">'R08 GL account map'!$4:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'R09 Payees'!$A$4:$L$15</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="13">'R09 Payees'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'R11 Receipt series in use'!$A$4:$L$12</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="14">'R11 Receipt series in use'!$4:$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'R11 Receipt series'!$A$4:$L$12</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="14">'R11 Receipt series'!$4:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'C01 Client master'!$A$4:$L$40</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="15">'C01 Client master'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'C02 Client addresses and'!$A$4:$L$17</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="16">'C02 Client addresses and'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'C03 Client payout accounts'!$A$4:$L$10</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="17">'C03 Client payout accounts'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'P01 In-force policy headers'!$A$4:$L$33</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="18">'P01 In-force policy headers'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'P01S Policy insurer shares'!$A$4:$L$10</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="19">'P01S Policy insurer shares'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="20" hidden="1">'P03 RMEL cohorts already'!$A$4:$L$16</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="20">'P03 RMEL cohorts already'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="21" hidden="1">'F01 Invoices header'!$A$4:$L$42</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="21">'F01 Invoices header'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="22" hidden="1">'F01S Invoices insurer shares'!$A$4:$L$9</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="22">'F01S Invoices insurer shares'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="23" hidden="1">'F01C Invoices components and'!$A$4:$L$12</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="23">'F01C Invoices components and'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="24" hidden="1">'F02 Unapplied premium payments'!$A$4:$L$25</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="24">'F02 Unapplied premium payments'!$4:$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'C02 Client addresses'!$A$4:$L$17</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="16">'C02 Client addresses'!$4:$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'C03 Payout accounts'!$A$4:$L$10</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="17">'C03 Payout accounts'!$4:$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'P01 Policy headers'!$A$4:$L$33</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="18">'P01 Policy headers'!$4:$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'P01S Policy shares'!$A$4:$L$10</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="19">'P01S Policy shares'!$4:$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="20" hidden="1">'P03 RMEL cohorts'!$A$4:$L$16</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="20">'P03 RMEL cohorts'!$4:$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="21" hidden="1">'F01 Invoice header'!$A$4:$L$42</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="21">'F01 Invoice header'!$4:$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="22" hidden="1">'F01S Invoice shares'!$A$4:$L$9</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="22">'F01S Invoice shares'!$4:$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="23" hidden="1">'F01C Invoice components'!$A$4:$L$12</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="23">'F01C Invoice components'!$4:$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="24" hidden="1">'F02 UPP'!$A$4:$L$25</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="24">'F02 UPP'!$4:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="25" hidden="1">'F03 Open collection state'!$A$4:$L$16</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="25">'F03 Open collection state'!$4:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="26" hidden="1">'F04 Remittance in flight'!$A$4:$L$14</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="26">'F04 Remittance in flight'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="27" hidden="1">'F06 PDCs, check pick-ups and'!$A$4:$L$18</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="27">'F06 PDCs, check pick-ups and'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="28" hidden="1">'G01 GL opening trial balance'!$A$4:$L$14</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="28">'G01 GL opening trial balance'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="29" hidden="1">'H01 Archive records closed'!$A$4:$L$19</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="29">'H01 Archive records closed'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="30" hidden="1">'H02 Archive documents index'!$A$4:$L$12</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="30">'H02 Archive documents index'!$4:$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="27" hidden="1">'F06 PDCs pick-ups refunds'!$A$4:$L$18</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="27">'F06 PDCs pick-ups refunds'!$4:$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="28" hidden="1">'G01 GL trial balance'!$A$4:$L$14</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="28">'G01 GL trial balance'!$4:$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="29" hidden="1">'H01 Archive records'!$A$4:$L$19</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="29">'H01 Archive records'!$4:$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="30" hidden="1">'H02 Archive documents'!$A$4:$L$12</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="30">'H02 Archive documents'!$4:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="31" hidden="1">'Control File'!$A$4:$L$16</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="31">'Control File'!$4:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="32" hidden="1">'Control Example'!$A$4:$L$11</definedName>
@@ -1020,7 +1020,7 @@
     <row r="23">
       <c r="B23" s="13" t="inlineStr">
         <is>
-          <t>R01 Lists of values and MIS</t>
+          <t>R01 LOV and MIS values</t>
         </is>
       </c>
       <c r="C23" s="14" t="inlineStr">
@@ -1035,7 +1035,7 @@
     <row r="24">
       <c r="B24" s="11" t="inlineStr">
         <is>
-          <t>R02 Branches and invoicing</t>
+          <t>R02 Branches</t>
         </is>
       </c>
       <c r="C24" s="12" t="inlineStr">
@@ -1050,7 +1050,7 @@
     <row r="25">
       <c r="B25" s="13" t="inlineStr">
         <is>
-          <t>R03 Sales organisation units</t>
+          <t>R03 Sales organisation</t>
         </is>
       </c>
       <c r="C25" s="14" t="inlineStr">
@@ -1095,7 +1095,7 @@
     <row r="28">
       <c r="B28" s="11" t="inlineStr">
         <is>
-          <t>R05 Product lines, cover types,</t>
+          <t>R05 Products and risk codes</t>
         </is>
       </c>
       <c r="C28" s="12" t="inlineStr">
@@ -1110,7 +1110,7 @@
     <row r="29">
       <c r="B29" s="13" t="inlineStr">
         <is>
-          <t>R06 Packages active versions</t>
+          <t>R06 Packages</t>
         </is>
       </c>
       <c r="C29" s="14" t="inlineStr">
@@ -1125,7 +1125,7 @@
     <row r="30">
       <c r="B30" s="11" t="inlineStr">
         <is>
-          <t>R07 Commission rates by insurer</t>
+          <t>R07 Commission rates</t>
         </is>
       </c>
       <c r="C30" s="12" t="inlineStr">
@@ -1140,7 +1140,7 @@
     <row r="31">
       <c r="B31" s="13" t="inlineStr">
         <is>
-          <t>R08 Chart of accounts mapping</t>
+          <t>R08 GL account map</t>
         </is>
       </c>
       <c r="C31" s="14" t="inlineStr">
@@ -1170,7 +1170,7 @@
     <row r="33">
       <c r="B33" s="13" t="inlineStr">
         <is>
-          <t>R11 Receipt series in use</t>
+          <t>R11 Receipt series</t>
         </is>
       </c>
       <c r="C33" s="14" t="inlineStr">
@@ -1200,7 +1200,7 @@
     <row r="35">
       <c r="B35" s="13" t="inlineStr">
         <is>
-          <t>C02 Client addresses and</t>
+          <t>C02 Client addresses</t>
         </is>
       </c>
       <c r="C35" s="14" t="inlineStr">
@@ -1215,7 +1215,7 @@
     <row r="36">
       <c r="B36" s="11" t="inlineStr">
         <is>
-          <t>C03 Client payout accounts</t>
+          <t>C03 Payout accounts</t>
         </is>
       </c>
       <c r="C36" s="12" t="inlineStr">
@@ -1230,7 +1230,7 @@
     <row r="37">
       <c r="B37" s="13" t="inlineStr">
         <is>
-          <t>P01 In-force policy headers</t>
+          <t>P01 Policy headers</t>
         </is>
       </c>
       <c r="C37" s="14" t="inlineStr">
@@ -1245,7 +1245,7 @@
     <row r="38">
       <c r="B38" s="11" t="inlineStr">
         <is>
-          <t>P01S Policy insurer shares</t>
+          <t>P01S Policy shares</t>
         </is>
       </c>
       <c r="C38" s="12" t="inlineStr">
@@ -1260,7 +1260,7 @@
     <row r="39">
       <c r="B39" s="13" t="inlineStr">
         <is>
-          <t>P03 RMEL cohorts already</t>
+          <t>P03 RMEL cohorts</t>
         </is>
       </c>
       <c r="C39" s="14" t="inlineStr">
@@ -1275,7 +1275,7 @@
     <row r="40">
       <c r="B40" s="11" t="inlineStr">
         <is>
-          <t>F01 Invoices header</t>
+          <t>F01 Invoice header</t>
         </is>
       </c>
       <c r="C40" s="12" t="inlineStr">
@@ -1290,7 +1290,7 @@
     <row r="41">
       <c r="B41" s="13" t="inlineStr">
         <is>
-          <t>F01S Invoices insurer shares</t>
+          <t>F01S Invoice shares</t>
         </is>
       </c>
       <c r="C41" s="14" t="inlineStr">
@@ -1305,7 +1305,7 @@
     <row r="42">
       <c r="B42" s="11" t="inlineStr">
         <is>
-          <t>F01C Invoices components and</t>
+          <t>F01C Invoice components</t>
         </is>
       </c>
       <c r="C42" s="12" t="inlineStr">
@@ -1320,7 +1320,7 @@
     <row r="43">
       <c r="B43" s="13" t="inlineStr">
         <is>
-          <t>F02 Unapplied premium payments</t>
+          <t>F02 UPP</t>
         </is>
       </c>
       <c r="C43" s="14" t="inlineStr">
@@ -1365,7 +1365,7 @@
     <row r="46">
       <c r="B46" s="11" t="inlineStr">
         <is>
-          <t>F06 PDCs, check pick-ups and</t>
+          <t>F06 PDCs pick-ups refunds</t>
         </is>
       </c>
       <c r="C46" s="12" t="inlineStr">
@@ -1380,7 +1380,7 @@
     <row r="47">
       <c r="B47" s="13" t="inlineStr">
         <is>
-          <t>G01 GL opening trial balance</t>
+          <t>G01 GL trial balance</t>
         </is>
       </c>
       <c r="C47" s="14" t="inlineStr">
@@ -1395,7 +1395,7 @@
     <row r="48">
       <c r="B48" s="11" t="inlineStr">
         <is>
-          <t>H01 Archive records closed</t>
+          <t>H01 Archive records</t>
         </is>
       </c>
       <c r="C48" s="12" t="inlineStr">
@@ -1410,7 +1410,7 @@
     <row r="49">
       <c r="B49" s="13" t="inlineStr">
         <is>
-          <t>H02 Archive documents index</t>
+          <t>H02 Archive documents</t>
         </is>
       </c>
       <c r="C49" s="14" t="inlineStr">
@@ -1707,7 +1707,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="21" t="inlineStr">
         <is>
-          <t>R05 Product lines, cover types,</t>
+          <t>R05 Products and risk codes</t>
         </is>
       </c>
     </row>
@@ -2392,7 +2392,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="21" t="inlineStr">
         <is>
-          <t>R06 Packages active versions</t>
+          <t>R06 Packages</t>
         </is>
       </c>
     </row>
@@ -3137,7 +3137,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="21" t="inlineStr">
         <is>
-          <t>R07 Commission rates by insurer</t>
+          <t>R07 Commission rates</t>
         </is>
       </c>
     </row>
@@ -3582,7 +3582,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="21" t="inlineStr">
         <is>
-          <t>R08 Chart of accounts mapping</t>
+          <t>R08 GL account map</t>
         </is>
       </c>
     </row>
@@ -5012,7 +5012,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="21" t="inlineStr">
         <is>
-          <t>R11 Receipt series in use</t>
+          <t>R11 Receipt series</t>
         </is>
       </c>
     </row>
@@ -7941,7 +7941,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="21" t="inlineStr">
         <is>
-          <t>C02 Client addresses and</t>
+          <t>C02 Client addresses</t>
         </is>
       </c>
     </row>
@@ -8866,7 +8866,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="21" t="inlineStr">
         <is>
-          <t>C03 Client payout accounts</t>
+          <t>C03 Payout accounts</t>
         </is>
       </c>
     </row>
@@ -9371,7 +9371,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="21" t="inlineStr">
         <is>
-          <t>P01 In-force policy headers</t>
+          <t>P01 Policy headers</t>
         </is>
       </c>
     </row>
@@ -11692,7 +11692,7 @@
     <row r="27">
       <c r="A27" s="12" t="inlineStr">
         <is>
-          <t>R01 Lists of values and MIS</t>
+          <t>R01 LOV and MIS values</t>
         </is>
       </c>
       <c r="B27" s="22" t="inlineStr">
@@ -11710,7 +11710,7 @@
     <row r="28">
       <c r="A28" s="14" t="inlineStr">
         <is>
-          <t>R01 Lists of values and MIS</t>
+          <t>R01 LOV and MIS values</t>
         </is>
       </c>
       <c r="B28" s="23" t="inlineStr">
@@ -11728,7 +11728,7 @@
     <row r="29">
       <c r="A29" s="12" t="inlineStr">
         <is>
-          <t>R01 Lists of values and MIS</t>
+          <t>R01 LOV and MIS values</t>
         </is>
       </c>
       <c r="B29" s="22" t="inlineStr">
@@ -11746,7 +11746,7 @@
     <row r="30">
       <c r="A30" s="14" t="inlineStr">
         <is>
-          <t>R01 Lists of values and MIS</t>
+          <t>R01 LOV and MIS values</t>
         </is>
       </c>
       <c r="B30" s="23" t="inlineStr">
@@ -11768,7 +11768,7 @@
     <row r="31">
       <c r="A31" s="12" t="inlineStr">
         <is>
-          <t>R01 Lists of values and MIS</t>
+          <t>R01 LOV and MIS values</t>
         </is>
       </c>
       <c r="B31" s="22" t="inlineStr">
@@ -11786,7 +11786,7 @@
     <row r="32">
       <c r="A32" s="14" t="inlineStr">
         <is>
-          <t>R01 Lists of values and MIS</t>
+          <t>R01 LOV and MIS values</t>
         </is>
       </c>
       <c r="B32" s="23" t="inlineStr">
@@ -11808,7 +11808,7 @@
     <row r="33">
       <c r="A33" s="12" t="inlineStr">
         <is>
-          <t>R01 Lists of values and MIS</t>
+          <t>R01 LOV and MIS values</t>
         </is>
       </c>
       <c r="B33" s="22" t="inlineStr">
@@ -11826,7 +11826,7 @@
     <row r="34">
       <c r="A34" s="14" t="inlineStr">
         <is>
-          <t>R01 Lists of values and MIS</t>
+          <t>R01 LOV and MIS values</t>
         </is>
       </c>
       <c r="B34" s="23" t="inlineStr">
@@ -11844,7 +11844,7 @@
     <row r="35">
       <c r="A35" s="12" t="inlineStr">
         <is>
-          <t>R01 Lists of values and MIS</t>
+          <t>R01 LOV and MIS values</t>
         </is>
       </c>
       <c r="B35" s="22" t="inlineStr">
@@ -11862,7 +11862,7 @@
     <row r="36">
       <c r="A36" s="14" t="inlineStr">
         <is>
-          <t>R01 Lists of values and MIS</t>
+          <t>R01 LOV and MIS values</t>
         </is>
       </c>
       <c r="B36" s="23" t="inlineStr">
@@ -11880,7 +11880,7 @@
     <row r="37">
       <c r="A37" s="12" t="inlineStr">
         <is>
-          <t>R01 Lists of values and MIS</t>
+          <t>R01 LOV and MIS values</t>
         </is>
       </c>
       <c r="B37" s="22" t="inlineStr">
@@ -11898,7 +11898,7 @@
     <row r="38">
       <c r="A38" s="14" t="inlineStr">
         <is>
-          <t>R01 Lists of values and MIS</t>
+          <t>R01 LOV and MIS values</t>
         </is>
       </c>
       <c r="B38" s="23" t="inlineStr">
@@ -11916,7 +11916,7 @@
     <row r="39">
       <c r="A39" s="12" t="inlineStr">
         <is>
-          <t>R02 Branches and invoicing</t>
+          <t>R02 Branches</t>
         </is>
       </c>
       <c r="B39" s="22" t="inlineStr">
@@ -11934,7 +11934,7 @@
     <row r="40">
       <c r="A40" s="14" t="inlineStr">
         <is>
-          <t>R02 Branches and invoicing</t>
+          <t>R02 Branches</t>
         </is>
       </c>
       <c r="B40" s="23" t="inlineStr">
@@ -11952,7 +11952,7 @@
     <row r="41">
       <c r="A41" s="12" t="inlineStr">
         <is>
-          <t>R02 Branches and invoicing</t>
+          <t>R02 Branches</t>
         </is>
       </c>
       <c r="B41" s="22" t="inlineStr">
@@ -11970,7 +11970,7 @@
     <row r="42">
       <c r="A42" s="14" t="inlineStr">
         <is>
-          <t>R02 Branches and invoicing</t>
+          <t>R02 Branches</t>
         </is>
       </c>
       <c r="B42" s="23" t="inlineStr">
@@ -11992,7 +11992,7 @@
     <row r="43">
       <c r="A43" s="12" t="inlineStr">
         <is>
-          <t>R02 Branches and invoicing</t>
+          <t>R02 Branches</t>
         </is>
       </c>
       <c r="B43" s="22" t="inlineStr">
@@ -12010,7 +12010,7 @@
     <row r="44">
       <c r="A44" s="14" t="inlineStr">
         <is>
-          <t>R02 Branches and invoicing</t>
+          <t>R02 Branches</t>
         </is>
       </c>
       <c r="B44" s="23" t="inlineStr">
@@ -12032,7 +12032,7 @@
     <row r="45">
       <c r="A45" s="12" t="inlineStr">
         <is>
-          <t>R02 Branches and invoicing</t>
+          <t>R02 Branches</t>
         </is>
       </c>
       <c r="B45" s="22" t="inlineStr">
@@ -12050,7 +12050,7 @@
     <row r="46">
       <c r="A46" s="14" t="inlineStr">
         <is>
-          <t>R02 Branches and invoicing</t>
+          <t>R02 Branches</t>
         </is>
       </c>
       <c r="B46" s="23" t="inlineStr">
@@ -12068,7 +12068,7 @@
     <row r="47">
       <c r="A47" s="12" t="inlineStr">
         <is>
-          <t>R02 Branches and invoicing</t>
+          <t>R02 Branches</t>
         </is>
       </c>
       <c r="B47" s="22" t="inlineStr">
@@ -12086,7 +12086,7 @@
     <row r="48">
       <c r="A48" s="14" t="inlineStr">
         <is>
-          <t>R02 Branches and invoicing</t>
+          <t>R02 Branches</t>
         </is>
       </c>
       <c r="B48" s="23" t="inlineStr">
@@ -12104,7 +12104,7 @@
     <row r="49">
       <c r="A49" s="12" t="inlineStr">
         <is>
-          <t>R02 Branches and invoicing</t>
+          <t>R02 Branches</t>
         </is>
       </c>
       <c r="B49" s="22" t="inlineStr">
@@ -12122,7 +12122,7 @@
     <row r="50">
       <c r="A50" s="14" t="inlineStr">
         <is>
-          <t>R02 Branches and invoicing</t>
+          <t>R02 Branches</t>
         </is>
       </c>
       <c r="B50" s="23" t="inlineStr">
@@ -12140,7 +12140,7 @@
     <row r="51">
       <c r="A51" s="12" t="inlineStr">
         <is>
-          <t>R03 Sales organisation units</t>
+          <t>R03 Sales organisation</t>
         </is>
       </c>
       <c r="B51" s="22" t="inlineStr">
@@ -12158,7 +12158,7 @@
     <row r="52">
       <c r="A52" s="14" t="inlineStr">
         <is>
-          <t>R03 Sales organisation units</t>
+          <t>R03 Sales organisation</t>
         </is>
       </c>
       <c r="B52" s="23" t="inlineStr">
@@ -12176,7 +12176,7 @@
     <row r="53">
       <c r="A53" s="12" t="inlineStr">
         <is>
-          <t>R03 Sales organisation units</t>
+          <t>R03 Sales organisation</t>
         </is>
       </c>
       <c r="B53" s="22" t="inlineStr">
@@ -12194,7 +12194,7 @@
     <row r="54">
       <c r="A54" s="14" t="inlineStr">
         <is>
-          <t>R03 Sales organisation units</t>
+          <t>R03 Sales organisation</t>
         </is>
       </c>
       <c r="B54" s="23" t="inlineStr">
@@ -12216,7 +12216,7 @@
     <row r="55">
       <c r="A55" s="12" t="inlineStr">
         <is>
-          <t>R03 Sales organisation units</t>
+          <t>R03 Sales organisation</t>
         </is>
       </c>
       <c r="B55" s="22" t="inlineStr">
@@ -12234,7 +12234,7 @@
     <row r="56">
       <c r="A56" s="14" t="inlineStr">
         <is>
-          <t>R03 Sales organisation units</t>
+          <t>R03 Sales organisation</t>
         </is>
       </c>
       <c r="B56" s="23" t="inlineStr">
@@ -12256,7 +12256,7 @@
     <row r="57">
       <c r="A57" s="12" t="inlineStr">
         <is>
-          <t>R03 Sales organisation units</t>
+          <t>R03 Sales organisation</t>
         </is>
       </c>
       <c r="B57" s="22" t="inlineStr">
@@ -12274,7 +12274,7 @@
     <row r="58">
       <c r="A58" s="14" t="inlineStr">
         <is>
-          <t>R03 Sales organisation units</t>
+          <t>R03 Sales organisation</t>
         </is>
       </c>
       <c r="B58" s="23" t="inlineStr">
@@ -12292,7 +12292,7 @@
     <row r="59">
       <c r="A59" s="12" t="inlineStr">
         <is>
-          <t>R03 Sales organisation units</t>
+          <t>R03 Sales organisation</t>
         </is>
       </c>
       <c r="B59" s="22" t="inlineStr">
@@ -12310,7 +12310,7 @@
     <row r="60">
       <c r="A60" s="14" t="inlineStr">
         <is>
-          <t>R03 Sales organisation units</t>
+          <t>R03 Sales organisation</t>
         </is>
       </c>
       <c r="B60" s="23" t="inlineStr">
@@ -12328,7 +12328,7 @@
     <row r="61">
       <c r="A61" s="12" t="inlineStr">
         <is>
-          <t>R03 Sales organisation units</t>
+          <t>R03 Sales organisation</t>
         </is>
       </c>
       <c r="B61" s="22" t="inlineStr">
@@ -12346,7 +12346,7 @@
     <row r="62">
       <c r="A62" s="14" t="inlineStr">
         <is>
-          <t>R03 Sales organisation units</t>
+          <t>R03 Sales organisation</t>
         </is>
       </c>
       <c r="B62" s="23" t="inlineStr">
@@ -12812,7 +12812,7 @@
     <row r="87">
       <c r="A87" s="12" t="inlineStr">
         <is>
-          <t>R05 Product lines, cover types,</t>
+          <t>R05 Products and risk codes</t>
         </is>
       </c>
       <c r="B87" s="22" t="inlineStr">
@@ -12830,7 +12830,7 @@
     <row r="88">
       <c r="A88" s="14" t="inlineStr">
         <is>
-          <t>R05 Product lines, cover types,</t>
+          <t>R05 Products and risk codes</t>
         </is>
       </c>
       <c r="B88" s="23" t="inlineStr">
@@ -12848,7 +12848,7 @@
     <row r="89">
       <c r="A89" s="12" t="inlineStr">
         <is>
-          <t>R05 Product lines, cover types,</t>
+          <t>R05 Products and risk codes</t>
         </is>
       </c>
       <c r="B89" s="22" t="inlineStr">
@@ -12866,7 +12866,7 @@
     <row r="90">
       <c r="A90" s="14" t="inlineStr">
         <is>
-          <t>R05 Product lines, cover types,</t>
+          <t>R05 Products and risk codes</t>
         </is>
       </c>
       <c r="B90" s="23" t="inlineStr">
@@ -12888,7 +12888,7 @@
     <row r="91">
       <c r="A91" s="12" t="inlineStr">
         <is>
-          <t>R05 Product lines, cover types,</t>
+          <t>R05 Products and risk codes</t>
         </is>
       </c>
       <c r="B91" s="22" t="inlineStr">
@@ -12906,7 +12906,7 @@
     <row r="92">
       <c r="A92" s="14" t="inlineStr">
         <is>
-          <t>R05 Product lines, cover types,</t>
+          <t>R05 Products and risk codes</t>
         </is>
       </c>
       <c r="B92" s="23" t="inlineStr">
@@ -12928,7 +12928,7 @@
     <row r="93">
       <c r="A93" s="12" t="inlineStr">
         <is>
-          <t>R05 Product lines, cover types,</t>
+          <t>R05 Products and risk codes</t>
         </is>
       </c>
       <c r="B93" s="22" t="inlineStr">
@@ -12946,7 +12946,7 @@
     <row r="94">
       <c r="A94" s="14" t="inlineStr">
         <is>
-          <t>R05 Product lines, cover types,</t>
+          <t>R05 Products and risk codes</t>
         </is>
       </c>
       <c r="B94" s="23" t="inlineStr">
@@ -12964,7 +12964,7 @@
     <row r="95">
       <c r="A95" s="12" t="inlineStr">
         <is>
-          <t>R05 Product lines, cover types,</t>
+          <t>R05 Products and risk codes</t>
         </is>
       </c>
       <c r="B95" s="22" t="inlineStr">
@@ -12982,7 +12982,7 @@
     <row r="96">
       <c r="A96" s="14" t="inlineStr">
         <is>
-          <t>R05 Product lines, cover types,</t>
+          <t>R05 Products and risk codes</t>
         </is>
       </c>
       <c r="B96" s="23" t="inlineStr">
@@ -13000,7 +13000,7 @@
     <row r="97">
       <c r="A97" s="12" t="inlineStr">
         <is>
-          <t>R05 Product lines, cover types,</t>
+          <t>R05 Products and risk codes</t>
         </is>
       </c>
       <c r="B97" s="22" t="inlineStr">
@@ -13018,7 +13018,7 @@
     <row r="98">
       <c r="A98" s="14" t="inlineStr">
         <is>
-          <t>R05 Product lines, cover types,</t>
+          <t>R05 Products and risk codes</t>
         </is>
       </c>
       <c r="B98" s="23" t="inlineStr">
@@ -13036,7 +13036,7 @@
     <row r="99">
       <c r="A99" s="12" t="inlineStr">
         <is>
-          <t>R06 Packages active versions</t>
+          <t>R06 Packages</t>
         </is>
       </c>
       <c r="B99" s="22" t="inlineStr">
@@ -13054,7 +13054,7 @@
     <row r="100">
       <c r="A100" s="14" t="inlineStr">
         <is>
-          <t>R06 Packages active versions</t>
+          <t>R06 Packages</t>
         </is>
       </c>
       <c r="B100" s="23" t="inlineStr">
@@ -13072,7 +13072,7 @@
     <row r="101">
       <c r="A101" s="12" t="inlineStr">
         <is>
-          <t>R06 Packages active versions</t>
+          <t>R06 Packages</t>
         </is>
       </c>
       <c r="B101" s="22" t="inlineStr">
@@ -13090,7 +13090,7 @@
     <row r="102">
       <c r="A102" s="14" t="inlineStr">
         <is>
-          <t>R06 Packages active versions</t>
+          <t>R06 Packages</t>
         </is>
       </c>
       <c r="B102" s="23" t="inlineStr">
@@ -13112,7 +13112,7 @@
     <row r="103">
       <c r="A103" s="12" t="inlineStr">
         <is>
-          <t>R06 Packages active versions</t>
+          <t>R06 Packages</t>
         </is>
       </c>
       <c r="B103" s="22" t="inlineStr">
@@ -13130,7 +13130,7 @@
     <row r="104">
       <c r="A104" s="14" t="inlineStr">
         <is>
-          <t>R06 Packages active versions</t>
+          <t>R06 Packages</t>
         </is>
       </c>
       <c r="B104" s="23" t="inlineStr">
@@ -13152,7 +13152,7 @@
     <row r="105">
       <c r="A105" s="12" t="inlineStr">
         <is>
-          <t>R06 Packages active versions</t>
+          <t>R06 Packages</t>
         </is>
       </c>
       <c r="B105" s="22" t="inlineStr">
@@ -13170,7 +13170,7 @@
     <row r="106">
       <c r="A106" s="14" t="inlineStr">
         <is>
-          <t>R06 Packages active versions</t>
+          <t>R06 Packages</t>
         </is>
       </c>
       <c r="B106" s="23" t="inlineStr">
@@ -13188,7 +13188,7 @@
     <row r="107">
       <c r="A107" s="12" t="inlineStr">
         <is>
-          <t>R06 Packages active versions</t>
+          <t>R06 Packages</t>
         </is>
       </c>
       <c r="B107" s="22" t="inlineStr">
@@ -13206,7 +13206,7 @@
     <row r="108">
       <c r="A108" s="14" t="inlineStr">
         <is>
-          <t>R06 Packages active versions</t>
+          <t>R06 Packages</t>
         </is>
       </c>
       <c r="B108" s="23" t="inlineStr">
@@ -13224,7 +13224,7 @@
     <row r="109">
       <c r="A109" s="12" t="inlineStr">
         <is>
-          <t>R06 Packages active versions</t>
+          <t>R06 Packages</t>
         </is>
       </c>
       <c r="B109" s="22" t="inlineStr">
@@ -13242,7 +13242,7 @@
     <row r="110">
       <c r="A110" s="14" t="inlineStr">
         <is>
-          <t>R06 Packages active versions</t>
+          <t>R06 Packages</t>
         </is>
       </c>
       <c r="B110" s="23" t="inlineStr">
@@ -13260,7 +13260,7 @@
     <row r="111">
       <c r="A111" s="12" t="inlineStr">
         <is>
-          <t>R07 Commission rates by insurer</t>
+          <t>R07 Commission rates</t>
         </is>
       </c>
       <c r="B111" s="22" t="inlineStr">
@@ -13278,7 +13278,7 @@
     <row r="112">
       <c r="A112" s="14" t="inlineStr">
         <is>
-          <t>R07 Commission rates by insurer</t>
+          <t>R07 Commission rates</t>
         </is>
       </c>
       <c r="B112" s="23" t="inlineStr">
@@ -13296,7 +13296,7 @@
     <row r="113">
       <c r="A113" s="12" t="inlineStr">
         <is>
-          <t>R07 Commission rates by insurer</t>
+          <t>R07 Commission rates</t>
         </is>
       </c>
       <c r="B113" s="22" t="inlineStr">
@@ -13314,7 +13314,7 @@
     <row r="114">
       <c r="A114" s="14" t="inlineStr">
         <is>
-          <t>R07 Commission rates by insurer</t>
+          <t>R07 Commission rates</t>
         </is>
       </c>
       <c r="B114" s="23" t="inlineStr">
@@ -13336,7 +13336,7 @@
     <row r="115">
       <c r="A115" s="12" t="inlineStr">
         <is>
-          <t>R07 Commission rates by insurer</t>
+          <t>R07 Commission rates</t>
         </is>
       </c>
       <c r="B115" s="22" t="inlineStr">
@@ -13354,7 +13354,7 @@
     <row r="116">
       <c r="A116" s="14" t="inlineStr">
         <is>
-          <t>R07 Commission rates by insurer</t>
+          <t>R07 Commission rates</t>
         </is>
       </c>
       <c r="B116" s="23" t="inlineStr">
@@ -13376,7 +13376,7 @@
     <row r="117">
       <c r="A117" s="12" t="inlineStr">
         <is>
-          <t>R07 Commission rates by insurer</t>
+          <t>R07 Commission rates</t>
         </is>
       </c>
       <c r="B117" s="22" t="inlineStr">
@@ -13394,7 +13394,7 @@
     <row r="118">
       <c r="A118" s="14" t="inlineStr">
         <is>
-          <t>R07 Commission rates by insurer</t>
+          <t>R07 Commission rates</t>
         </is>
       </c>
       <c r="B118" s="23" t="inlineStr">
@@ -13412,7 +13412,7 @@
     <row r="119">
       <c r="A119" s="12" t="inlineStr">
         <is>
-          <t>R07 Commission rates by insurer</t>
+          <t>R07 Commission rates</t>
         </is>
       </c>
       <c r="B119" s="22" t="inlineStr">
@@ -13430,7 +13430,7 @@
     <row r="120">
       <c r="A120" s="14" t="inlineStr">
         <is>
-          <t>R07 Commission rates by insurer</t>
+          <t>R07 Commission rates</t>
         </is>
       </c>
       <c r="B120" s="23" t="inlineStr">
@@ -13448,7 +13448,7 @@
     <row r="121">
       <c r="A121" s="12" t="inlineStr">
         <is>
-          <t>R07 Commission rates by insurer</t>
+          <t>R07 Commission rates</t>
         </is>
       </c>
       <c r="B121" s="22" t="inlineStr">
@@ -13466,7 +13466,7 @@
     <row r="122">
       <c r="A122" s="14" t="inlineStr">
         <is>
-          <t>R07 Commission rates by insurer</t>
+          <t>R07 Commission rates</t>
         </is>
       </c>
       <c r="B122" s="23" t="inlineStr">
@@ -13484,7 +13484,7 @@
     <row r="123">
       <c r="A123" s="12" t="inlineStr">
         <is>
-          <t>R08 Chart of accounts mapping</t>
+          <t>R08 GL account map</t>
         </is>
       </c>
       <c r="B123" s="22" t="inlineStr">
@@ -13502,7 +13502,7 @@
     <row r="124">
       <c r="A124" s="14" t="inlineStr">
         <is>
-          <t>R08 Chart of accounts mapping</t>
+          <t>R08 GL account map</t>
         </is>
       </c>
       <c r="B124" s="23" t="inlineStr">
@@ -13520,7 +13520,7 @@
     <row r="125">
       <c r="A125" s="12" t="inlineStr">
         <is>
-          <t>R08 Chart of accounts mapping</t>
+          <t>R08 GL account map</t>
         </is>
       </c>
       <c r="B125" s="22" t="inlineStr">
@@ -13538,7 +13538,7 @@
     <row r="126">
       <c r="A126" s="14" t="inlineStr">
         <is>
-          <t>R08 Chart of accounts mapping</t>
+          <t>R08 GL account map</t>
         </is>
       </c>
       <c r="B126" s="23" t="inlineStr">
@@ -13560,7 +13560,7 @@
     <row r="127">
       <c r="A127" s="12" t="inlineStr">
         <is>
-          <t>R08 Chart of accounts mapping</t>
+          <t>R08 GL account map</t>
         </is>
       </c>
       <c r="B127" s="22" t="inlineStr">
@@ -13578,7 +13578,7 @@
     <row r="128">
       <c r="A128" s="14" t="inlineStr">
         <is>
-          <t>R08 Chart of accounts mapping</t>
+          <t>R08 GL account map</t>
         </is>
       </c>
       <c r="B128" s="23" t="inlineStr">
@@ -13600,7 +13600,7 @@
     <row r="129">
       <c r="A129" s="12" t="inlineStr">
         <is>
-          <t>R08 Chart of accounts mapping</t>
+          <t>R08 GL account map</t>
         </is>
       </c>
       <c r="B129" s="22" t="inlineStr">
@@ -13618,7 +13618,7 @@
     <row r="130">
       <c r="A130" s="14" t="inlineStr">
         <is>
-          <t>R08 Chart of accounts mapping</t>
+          <t>R08 GL account map</t>
         </is>
       </c>
       <c r="B130" s="23" t="inlineStr">
@@ -13636,7 +13636,7 @@
     <row r="131">
       <c r="A131" s="12" t="inlineStr">
         <is>
-          <t>R08 Chart of accounts mapping</t>
+          <t>R08 GL account map</t>
         </is>
       </c>
       <c r="B131" s="22" t="inlineStr">
@@ -13654,7 +13654,7 @@
     <row r="132">
       <c r="A132" s="14" t="inlineStr">
         <is>
-          <t>R08 Chart of accounts mapping</t>
+          <t>R08 GL account map</t>
         </is>
       </c>
       <c r="B132" s="23" t="inlineStr">
@@ -13672,7 +13672,7 @@
     <row r="133">
       <c r="A133" s="12" t="inlineStr">
         <is>
-          <t>R08 Chart of accounts mapping</t>
+          <t>R08 GL account map</t>
         </is>
       </c>
       <c r="B133" s="22" t="inlineStr">
@@ -13690,7 +13690,7 @@
     <row r="134">
       <c r="A134" s="14" t="inlineStr">
         <is>
-          <t>R08 Chart of accounts mapping</t>
+          <t>R08 GL account map</t>
         </is>
       </c>
       <c r="B134" s="23" t="inlineStr">
@@ -13932,7 +13932,7 @@
     <row r="147">
       <c r="A147" s="12" t="inlineStr">
         <is>
-          <t>R11 Receipt series in use</t>
+          <t>R11 Receipt series</t>
         </is>
       </c>
       <c r="B147" s="22" t="inlineStr">
@@ -13950,7 +13950,7 @@
     <row r="148">
       <c r="A148" s="14" t="inlineStr">
         <is>
-          <t>R11 Receipt series in use</t>
+          <t>R11 Receipt series</t>
         </is>
       </c>
       <c r="B148" s="23" t="inlineStr">
@@ -13968,7 +13968,7 @@
     <row r="149">
       <c r="A149" s="12" t="inlineStr">
         <is>
-          <t>R11 Receipt series in use</t>
+          <t>R11 Receipt series</t>
         </is>
       </c>
       <c r="B149" s="22" t="inlineStr">
@@ -13986,7 +13986,7 @@
     <row r="150">
       <c r="A150" s="14" t="inlineStr">
         <is>
-          <t>R11 Receipt series in use</t>
+          <t>R11 Receipt series</t>
         </is>
       </c>
       <c r="B150" s="23" t="inlineStr">
@@ -14008,7 +14008,7 @@
     <row r="151">
       <c r="A151" s="12" t="inlineStr">
         <is>
-          <t>R11 Receipt series in use</t>
+          <t>R11 Receipt series</t>
         </is>
       </c>
       <c r="B151" s="22" t="inlineStr">
@@ -14026,7 +14026,7 @@
     <row r="152">
       <c r="A152" s="14" t="inlineStr">
         <is>
-          <t>R11 Receipt series in use</t>
+          <t>R11 Receipt series</t>
         </is>
       </c>
       <c r="B152" s="23" t="inlineStr">
@@ -14048,7 +14048,7 @@
     <row r="153">
       <c r="A153" s="12" t="inlineStr">
         <is>
-          <t>R11 Receipt series in use</t>
+          <t>R11 Receipt series</t>
         </is>
       </c>
       <c r="B153" s="22" t="inlineStr">
@@ -14066,7 +14066,7 @@
     <row r="154">
       <c r="A154" s="14" t="inlineStr">
         <is>
-          <t>R11 Receipt series in use</t>
+          <t>R11 Receipt series</t>
         </is>
       </c>
       <c r="B154" s="23" t="inlineStr">
@@ -14084,7 +14084,7 @@
     <row r="155">
       <c r="A155" s="12" t="inlineStr">
         <is>
-          <t>R11 Receipt series in use</t>
+          <t>R11 Receipt series</t>
         </is>
       </c>
       <c r="B155" s="22" t="inlineStr">
@@ -14102,7 +14102,7 @@
     <row r="156">
       <c r="A156" s="14" t="inlineStr">
         <is>
-          <t>R11 Receipt series in use</t>
+          <t>R11 Receipt series</t>
         </is>
       </c>
       <c r="B156" s="23" t="inlineStr">
@@ -14120,7 +14120,7 @@
     <row r="157">
       <c r="A157" s="12" t="inlineStr">
         <is>
-          <t>R11 Receipt series in use</t>
+          <t>R11 Receipt series</t>
         </is>
       </c>
       <c r="B157" s="22" t="inlineStr">
@@ -14138,7 +14138,7 @@
     <row r="158">
       <c r="A158" s="14" t="inlineStr">
         <is>
-          <t>R11 Receipt series in use</t>
+          <t>R11 Receipt series</t>
         </is>
       </c>
       <c r="B158" s="23" t="inlineStr">
@@ -14380,7 +14380,7 @@
     <row r="171">
       <c r="A171" s="12" t="inlineStr">
         <is>
-          <t>C02 Client addresses and</t>
+          <t>C02 Client addresses</t>
         </is>
       </c>
       <c r="B171" s="22" t="inlineStr">
@@ -14398,7 +14398,7 @@
     <row r="172">
       <c r="A172" s="14" t="inlineStr">
         <is>
-          <t>C02 Client addresses and</t>
+          <t>C02 Client addresses</t>
         </is>
       </c>
       <c r="B172" s="23" t="inlineStr">
@@ -14416,7 +14416,7 @@
     <row r="173">
       <c r="A173" s="12" t="inlineStr">
         <is>
-          <t>C02 Client addresses and</t>
+          <t>C02 Client addresses</t>
         </is>
       </c>
       <c r="B173" s="22" t="inlineStr">
@@ -14434,7 +14434,7 @@
     <row r="174">
       <c r="A174" s="14" t="inlineStr">
         <is>
-          <t>C02 Client addresses and</t>
+          <t>C02 Client addresses</t>
         </is>
       </c>
       <c r="B174" s="23" t="inlineStr">
@@ -14456,7 +14456,7 @@
     <row r="175">
       <c r="A175" s="12" t="inlineStr">
         <is>
-          <t>C02 Client addresses and</t>
+          <t>C02 Client addresses</t>
         </is>
       </c>
       <c r="B175" s="22" t="inlineStr">
@@ -14474,7 +14474,7 @@
     <row r="176">
       <c r="A176" s="14" t="inlineStr">
         <is>
-          <t>C02 Client addresses and</t>
+          <t>C02 Client addresses</t>
         </is>
       </c>
       <c r="B176" s="23" t="inlineStr">
@@ -14496,7 +14496,7 @@
     <row r="177">
       <c r="A177" s="12" t="inlineStr">
         <is>
-          <t>C02 Client addresses and</t>
+          <t>C02 Client addresses</t>
         </is>
       </c>
       <c r="B177" s="22" t="inlineStr">
@@ -14514,7 +14514,7 @@
     <row r="178">
       <c r="A178" s="14" t="inlineStr">
         <is>
-          <t>C02 Client addresses and</t>
+          <t>C02 Client addresses</t>
         </is>
       </c>
       <c r="B178" s="23" t="inlineStr">
@@ -14532,7 +14532,7 @@
     <row r="179">
       <c r="A179" s="12" t="inlineStr">
         <is>
-          <t>C02 Client addresses and</t>
+          <t>C02 Client addresses</t>
         </is>
       </c>
       <c r="B179" s="22" t="inlineStr">
@@ -14550,7 +14550,7 @@
     <row r="180">
       <c r="A180" s="14" t="inlineStr">
         <is>
-          <t>C02 Client addresses and</t>
+          <t>C02 Client addresses</t>
         </is>
       </c>
       <c r="B180" s="23" t="inlineStr">
@@ -14568,7 +14568,7 @@
     <row r="181">
       <c r="A181" s="12" t="inlineStr">
         <is>
-          <t>C02 Client addresses and</t>
+          <t>C02 Client addresses</t>
         </is>
       </c>
       <c r="B181" s="22" t="inlineStr">
@@ -14586,7 +14586,7 @@
     <row r="182">
       <c r="A182" s="14" t="inlineStr">
         <is>
-          <t>C02 Client addresses and</t>
+          <t>C02 Client addresses</t>
         </is>
       </c>
       <c r="B182" s="23" t="inlineStr">
@@ -14604,7 +14604,7 @@
     <row r="183">
       <c r="A183" s="12" t="inlineStr">
         <is>
-          <t>C03 Client payout accounts</t>
+          <t>C03 Payout accounts</t>
         </is>
       </c>
       <c r="B183" s="22" t="inlineStr">
@@ -14622,7 +14622,7 @@
     <row r="184">
       <c r="A184" s="14" t="inlineStr">
         <is>
-          <t>C03 Client payout accounts</t>
+          <t>C03 Payout accounts</t>
         </is>
       </c>
       <c r="B184" s="23" t="inlineStr">
@@ -14640,7 +14640,7 @@
     <row r="185">
       <c r="A185" s="12" t="inlineStr">
         <is>
-          <t>C03 Client payout accounts</t>
+          <t>C03 Payout accounts</t>
         </is>
       </c>
       <c r="B185" s="22" t="inlineStr">
@@ -14658,7 +14658,7 @@
     <row r="186">
       <c r="A186" s="14" t="inlineStr">
         <is>
-          <t>C03 Client payout accounts</t>
+          <t>C03 Payout accounts</t>
         </is>
       </c>
       <c r="B186" s="23" t="inlineStr">
@@ -14680,7 +14680,7 @@
     <row r="187">
       <c r="A187" s="12" t="inlineStr">
         <is>
-          <t>C03 Client payout accounts</t>
+          <t>C03 Payout accounts</t>
         </is>
       </c>
       <c r="B187" s="22" t="inlineStr">
@@ -14698,7 +14698,7 @@
     <row r="188">
       <c r="A188" s="14" t="inlineStr">
         <is>
-          <t>C03 Client payout accounts</t>
+          <t>C03 Payout accounts</t>
         </is>
       </c>
       <c r="B188" s="23" t="inlineStr">
@@ -14720,7 +14720,7 @@
     <row r="189">
       <c r="A189" s="12" t="inlineStr">
         <is>
-          <t>C03 Client payout accounts</t>
+          <t>C03 Payout accounts</t>
         </is>
       </c>
       <c r="B189" s="22" t="inlineStr">
@@ -14738,7 +14738,7 @@
     <row r="190">
       <c r="A190" s="14" t="inlineStr">
         <is>
-          <t>C03 Client payout accounts</t>
+          <t>C03 Payout accounts</t>
         </is>
       </c>
       <c r="B190" s="23" t="inlineStr">
@@ -14756,7 +14756,7 @@
     <row r="191">
       <c r="A191" s="12" t="inlineStr">
         <is>
-          <t>C03 Client payout accounts</t>
+          <t>C03 Payout accounts</t>
         </is>
       </c>
       <c r="B191" s="22" t="inlineStr">
@@ -14774,7 +14774,7 @@
     <row r="192">
       <c r="A192" s="14" t="inlineStr">
         <is>
-          <t>C03 Client payout accounts</t>
+          <t>C03 Payout accounts</t>
         </is>
       </c>
       <c r="B192" s="23" t="inlineStr">
@@ -14792,7 +14792,7 @@
     <row r="193">
       <c r="A193" s="12" t="inlineStr">
         <is>
-          <t>C03 Client payout accounts</t>
+          <t>C03 Payout accounts</t>
         </is>
       </c>
       <c r="B193" s="22" t="inlineStr">
@@ -14810,7 +14810,7 @@
     <row r="194">
       <c r="A194" s="14" t="inlineStr">
         <is>
-          <t>C03 Client payout accounts</t>
+          <t>C03 Payout accounts</t>
         </is>
       </c>
       <c r="B194" s="23" t="inlineStr">
@@ -14828,7 +14828,7 @@
     <row r="195">
       <c r="A195" s="12" t="inlineStr">
         <is>
-          <t>P01 In-force policy headers</t>
+          <t>P01 Policy headers</t>
         </is>
       </c>
       <c r="B195" s="22" t="inlineStr">
@@ -14846,7 +14846,7 @@
     <row r="196">
       <c r="A196" s="14" t="inlineStr">
         <is>
-          <t>P01 In-force policy headers</t>
+          <t>P01 Policy headers</t>
         </is>
       </c>
       <c r="B196" s="23" t="inlineStr">
@@ -14864,7 +14864,7 @@
     <row r="197">
       <c r="A197" s="12" t="inlineStr">
         <is>
-          <t>P01 In-force policy headers</t>
+          <t>P01 Policy headers</t>
         </is>
       </c>
       <c r="B197" s="22" t="inlineStr">
@@ -14882,7 +14882,7 @@
     <row r="198">
       <c r="A198" s="14" t="inlineStr">
         <is>
-          <t>P01 In-force policy headers</t>
+          <t>P01 Policy headers</t>
         </is>
       </c>
       <c r="B198" s="23" t="inlineStr">
@@ -14904,7 +14904,7 @@
     <row r="199">
       <c r="A199" s="12" t="inlineStr">
         <is>
-          <t>P01 In-force policy headers</t>
+          <t>P01 Policy headers</t>
         </is>
       </c>
       <c r="B199" s="22" t="inlineStr">
@@ -14922,7 +14922,7 @@
     <row r="200">
       <c r="A200" s="14" t="inlineStr">
         <is>
-          <t>P01 In-force policy headers</t>
+          <t>P01 Policy headers</t>
         </is>
       </c>
       <c r="B200" s="23" t="inlineStr">
@@ -14944,7 +14944,7 @@
     <row r="201">
       <c r="A201" s="12" t="inlineStr">
         <is>
-          <t>P01 In-force policy headers</t>
+          <t>P01 Policy headers</t>
         </is>
       </c>
       <c r="B201" s="22" t="inlineStr">
@@ -14962,7 +14962,7 @@
     <row r="202">
       <c r="A202" s="14" t="inlineStr">
         <is>
-          <t>P01 In-force policy headers</t>
+          <t>P01 Policy headers</t>
         </is>
       </c>
       <c r="B202" s="23" t="inlineStr">
@@ -14980,7 +14980,7 @@
     <row r="203">
       <c r="A203" s="12" t="inlineStr">
         <is>
-          <t>P01 In-force policy headers</t>
+          <t>P01 Policy headers</t>
         </is>
       </c>
       <c r="B203" s="22" t="inlineStr">
@@ -14998,7 +14998,7 @@
     <row r="204">
       <c r="A204" s="14" t="inlineStr">
         <is>
-          <t>P01 In-force policy headers</t>
+          <t>P01 Policy headers</t>
         </is>
       </c>
       <c r="B204" s="23" t="inlineStr">
@@ -15016,7 +15016,7 @@
     <row r="205">
       <c r="A205" s="12" t="inlineStr">
         <is>
-          <t>P01 In-force policy headers</t>
+          <t>P01 Policy headers</t>
         </is>
       </c>
       <c r="B205" s="22" t="inlineStr">
@@ -15034,7 +15034,7 @@
     <row r="206">
       <c r="A206" s="14" t="inlineStr">
         <is>
-          <t>P01 In-force policy headers</t>
+          <t>P01 Policy headers</t>
         </is>
       </c>
       <c r="B206" s="23" t="inlineStr">
@@ -15052,7 +15052,7 @@
     <row r="207">
       <c r="A207" s="12" t="inlineStr">
         <is>
-          <t>P01S Policy insurer shares</t>
+          <t>P01S Policy shares</t>
         </is>
       </c>
       <c r="B207" s="22" t="inlineStr">
@@ -15070,7 +15070,7 @@
     <row r="208">
       <c r="A208" s="14" t="inlineStr">
         <is>
-          <t>P01S Policy insurer shares</t>
+          <t>P01S Policy shares</t>
         </is>
       </c>
       <c r="B208" s="23" t="inlineStr">
@@ -15088,7 +15088,7 @@
     <row r="209">
       <c r="A209" s="12" t="inlineStr">
         <is>
-          <t>P01S Policy insurer shares</t>
+          <t>P01S Policy shares</t>
         </is>
       </c>
       <c r="B209" s="22" t="inlineStr">
@@ -15106,7 +15106,7 @@
     <row r="210">
       <c r="A210" s="14" t="inlineStr">
         <is>
-          <t>P01S Policy insurer shares</t>
+          <t>P01S Policy shares</t>
         </is>
       </c>
       <c r="B210" s="23" t="inlineStr">
@@ -15128,7 +15128,7 @@
     <row r="211">
       <c r="A211" s="12" t="inlineStr">
         <is>
-          <t>P01S Policy insurer shares</t>
+          <t>P01S Policy shares</t>
         </is>
       </c>
       <c r="B211" s="22" t="inlineStr">
@@ -15146,7 +15146,7 @@
     <row r="212">
       <c r="A212" s="14" t="inlineStr">
         <is>
-          <t>P01S Policy insurer shares</t>
+          <t>P01S Policy shares</t>
         </is>
       </c>
       <c r="B212" s="23" t="inlineStr">
@@ -15168,7 +15168,7 @@
     <row r="213">
       <c r="A213" s="12" t="inlineStr">
         <is>
-          <t>P01S Policy insurer shares</t>
+          <t>P01S Policy shares</t>
         </is>
       </c>
       <c r="B213" s="22" t="inlineStr">
@@ -15186,7 +15186,7 @@
     <row r="214">
       <c r="A214" s="14" t="inlineStr">
         <is>
-          <t>P01S Policy insurer shares</t>
+          <t>P01S Policy shares</t>
         </is>
       </c>
       <c r="B214" s="23" t="inlineStr">
@@ -15204,7 +15204,7 @@
     <row r="215">
       <c r="A215" s="12" t="inlineStr">
         <is>
-          <t>P01S Policy insurer shares</t>
+          <t>P01S Policy shares</t>
         </is>
       </c>
       <c r="B215" s="22" t="inlineStr">
@@ -15222,7 +15222,7 @@
     <row r="216">
       <c r="A216" s="14" t="inlineStr">
         <is>
-          <t>P01S Policy insurer shares</t>
+          <t>P01S Policy shares</t>
         </is>
       </c>
       <c r="B216" s="23" t="inlineStr">
@@ -15240,7 +15240,7 @@
     <row r="217">
       <c r="A217" s="12" t="inlineStr">
         <is>
-          <t>P01S Policy insurer shares</t>
+          <t>P01S Policy shares</t>
         </is>
       </c>
       <c r="B217" s="22" t="inlineStr">
@@ -15258,7 +15258,7 @@
     <row r="218">
       <c r="A218" s="14" t="inlineStr">
         <is>
-          <t>P01S Policy insurer shares</t>
+          <t>P01S Policy shares</t>
         </is>
       </c>
       <c r="B218" s="23" t="inlineStr">
@@ -15276,7 +15276,7 @@
     <row r="219">
       <c r="A219" s="12" t="inlineStr">
         <is>
-          <t>P03 RMEL cohorts already</t>
+          <t>P03 RMEL cohorts</t>
         </is>
       </c>
       <c r="B219" s="22" t="inlineStr">
@@ -15294,7 +15294,7 @@
     <row r="220">
       <c r="A220" s="14" t="inlineStr">
         <is>
-          <t>P03 RMEL cohorts already</t>
+          <t>P03 RMEL cohorts</t>
         </is>
       </c>
       <c r="B220" s="23" t="inlineStr">
@@ -15312,7 +15312,7 @@
     <row r="221">
       <c r="A221" s="12" t="inlineStr">
         <is>
-          <t>P03 RMEL cohorts already</t>
+          <t>P03 RMEL cohorts</t>
         </is>
       </c>
       <c r="B221" s="22" t="inlineStr">
@@ -15330,7 +15330,7 @@
     <row r="222">
       <c r="A222" s="14" t="inlineStr">
         <is>
-          <t>P03 RMEL cohorts already</t>
+          <t>P03 RMEL cohorts</t>
         </is>
       </c>
       <c r="B222" s="23" t="inlineStr">
@@ -15352,7 +15352,7 @@
     <row r="223">
       <c r="A223" s="12" t="inlineStr">
         <is>
-          <t>P03 RMEL cohorts already</t>
+          <t>P03 RMEL cohorts</t>
         </is>
       </c>
       <c r="B223" s="22" t="inlineStr">
@@ -15370,7 +15370,7 @@
     <row r="224">
       <c r="A224" s="14" t="inlineStr">
         <is>
-          <t>P03 RMEL cohorts already</t>
+          <t>P03 RMEL cohorts</t>
         </is>
       </c>
       <c r="B224" s="23" t="inlineStr">
@@ -15392,7 +15392,7 @@
     <row r="225">
       <c r="A225" s="12" t="inlineStr">
         <is>
-          <t>P03 RMEL cohorts already</t>
+          <t>P03 RMEL cohorts</t>
         </is>
       </c>
       <c r="B225" s="22" t="inlineStr">
@@ -15410,7 +15410,7 @@
     <row r="226">
       <c r="A226" s="14" t="inlineStr">
         <is>
-          <t>P03 RMEL cohorts already</t>
+          <t>P03 RMEL cohorts</t>
         </is>
       </c>
       <c r="B226" s="23" t="inlineStr">
@@ -15428,7 +15428,7 @@
     <row r="227">
       <c r="A227" s="12" t="inlineStr">
         <is>
-          <t>P03 RMEL cohorts already</t>
+          <t>P03 RMEL cohorts</t>
         </is>
       </c>
       <c r="B227" s="22" t="inlineStr">
@@ -15446,7 +15446,7 @@
     <row r="228">
       <c r="A228" s="14" t="inlineStr">
         <is>
-          <t>P03 RMEL cohorts already</t>
+          <t>P03 RMEL cohorts</t>
         </is>
       </c>
       <c r="B228" s="23" t="inlineStr">
@@ -15464,7 +15464,7 @@
     <row r="229">
       <c r="A229" s="12" t="inlineStr">
         <is>
-          <t>P03 RMEL cohorts already</t>
+          <t>P03 RMEL cohorts</t>
         </is>
       </c>
       <c r="B229" s="22" t="inlineStr">
@@ -15482,7 +15482,7 @@
     <row r="230">
       <c r="A230" s="14" t="inlineStr">
         <is>
-          <t>P03 RMEL cohorts already</t>
+          <t>P03 RMEL cohorts</t>
         </is>
       </c>
       <c r="B230" s="23" t="inlineStr">
@@ -15500,7 +15500,7 @@
     <row r="231">
       <c r="A231" s="12" t="inlineStr">
         <is>
-          <t>F01 Invoices header</t>
+          <t>F01 Invoice header</t>
         </is>
       </c>
       <c r="B231" s="22" t="inlineStr">
@@ -15518,7 +15518,7 @@
     <row r="232">
       <c r="A232" s="14" t="inlineStr">
         <is>
-          <t>F01 Invoices header</t>
+          <t>F01 Invoice header</t>
         </is>
       </c>
       <c r="B232" s="23" t="inlineStr">
@@ -15536,7 +15536,7 @@
     <row r="233">
       <c r="A233" s="12" t="inlineStr">
         <is>
-          <t>F01 Invoices header</t>
+          <t>F01 Invoice header</t>
         </is>
       </c>
       <c r="B233" s="22" t="inlineStr">
@@ -15554,7 +15554,7 @@
     <row r="234">
       <c r="A234" s="14" t="inlineStr">
         <is>
-          <t>F01 Invoices header</t>
+          <t>F01 Invoice header</t>
         </is>
       </c>
       <c r="B234" s="23" t="inlineStr">
@@ -15576,7 +15576,7 @@
     <row r="235">
       <c r="A235" s="12" t="inlineStr">
         <is>
-          <t>F01 Invoices header</t>
+          <t>F01 Invoice header</t>
         </is>
       </c>
       <c r="B235" s="22" t="inlineStr">
@@ -15594,7 +15594,7 @@
     <row r="236">
       <c r="A236" s="14" t="inlineStr">
         <is>
-          <t>F01 Invoices header</t>
+          <t>F01 Invoice header</t>
         </is>
       </c>
       <c r="B236" s="23" t="inlineStr">
@@ -15616,7 +15616,7 @@
     <row r="237">
       <c r="A237" s="12" t="inlineStr">
         <is>
-          <t>F01 Invoices header</t>
+          <t>F01 Invoice header</t>
         </is>
       </c>
       <c r="B237" s="22" t="inlineStr">
@@ -15634,7 +15634,7 @@
     <row r="238">
       <c r="A238" s="14" t="inlineStr">
         <is>
-          <t>F01 Invoices header</t>
+          <t>F01 Invoice header</t>
         </is>
       </c>
       <c r="B238" s="23" t="inlineStr">
@@ -15652,7 +15652,7 @@
     <row r="239">
       <c r="A239" s="12" t="inlineStr">
         <is>
-          <t>F01 Invoices header</t>
+          <t>F01 Invoice header</t>
         </is>
       </c>
       <c r="B239" s="22" t="inlineStr">
@@ -15670,7 +15670,7 @@
     <row r="240">
       <c r="A240" s="14" t="inlineStr">
         <is>
-          <t>F01 Invoices header</t>
+          <t>F01 Invoice header</t>
         </is>
       </c>
       <c r="B240" s="23" t="inlineStr">
@@ -15688,7 +15688,7 @@
     <row r="241">
       <c r="A241" s="12" t="inlineStr">
         <is>
-          <t>F01 Invoices header</t>
+          <t>F01 Invoice header</t>
         </is>
       </c>
       <c r="B241" s="22" t="inlineStr">
@@ -15706,7 +15706,7 @@
     <row r="242">
       <c r="A242" s="14" t="inlineStr">
         <is>
-          <t>F01 Invoices header</t>
+          <t>F01 Invoice header</t>
         </is>
       </c>
       <c r="B242" s="23" t="inlineStr">
@@ -15724,7 +15724,7 @@
     <row r="243">
       <c r="A243" s="12" t="inlineStr">
         <is>
-          <t>F01S Invoices insurer shares</t>
+          <t>F01S Invoice shares</t>
         </is>
       </c>
       <c r="B243" s="22" t="inlineStr">
@@ -15742,7 +15742,7 @@
     <row r="244">
       <c r="A244" s="14" t="inlineStr">
         <is>
-          <t>F01S Invoices insurer shares</t>
+          <t>F01S Invoice shares</t>
         </is>
       </c>
       <c r="B244" s="23" t="inlineStr">
@@ -15760,7 +15760,7 @@
     <row r="245">
       <c r="A245" s="12" t="inlineStr">
         <is>
-          <t>F01S Invoices insurer shares</t>
+          <t>F01S Invoice shares</t>
         </is>
       </c>
       <c r="B245" s="22" t="inlineStr">
@@ -15778,7 +15778,7 @@
     <row r="246">
       <c r="A246" s="14" t="inlineStr">
         <is>
-          <t>F01S Invoices insurer shares</t>
+          <t>F01S Invoice shares</t>
         </is>
       </c>
       <c r="B246" s="23" t="inlineStr">
@@ -15800,7 +15800,7 @@
     <row r="247">
       <c r="A247" s="12" t="inlineStr">
         <is>
-          <t>F01S Invoices insurer shares</t>
+          <t>F01S Invoice shares</t>
         </is>
       </c>
       <c r="B247" s="22" t="inlineStr">
@@ -15818,7 +15818,7 @@
     <row r="248">
       <c r="A248" s="14" t="inlineStr">
         <is>
-          <t>F01S Invoices insurer shares</t>
+          <t>F01S Invoice shares</t>
         </is>
       </c>
       <c r="B248" s="23" t="inlineStr">
@@ -15840,7 +15840,7 @@
     <row r="249">
       <c r="A249" s="12" t="inlineStr">
         <is>
-          <t>F01S Invoices insurer shares</t>
+          <t>F01S Invoice shares</t>
         </is>
       </c>
       <c r="B249" s="22" t="inlineStr">
@@ -15858,7 +15858,7 @@
     <row r="250">
       <c r="A250" s="14" t="inlineStr">
         <is>
-          <t>F01S Invoices insurer shares</t>
+          <t>F01S Invoice shares</t>
         </is>
       </c>
       <c r="B250" s="23" t="inlineStr">
@@ -15876,7 +15876,7 @@
     <row r="251">
       <c r="A251" s="12" t="inlineStr">
         <is>
-          <t>F01S Invoices insurer shares</t>
+          <t>F01S Invoice shares</t>
         </is>
       </c>
       <c r="B251" s="22" t="inlineStr">
@@ -15894,7 +15894,7 @@
     <row r="252">
       <c r="A252" s="14" t="inlineStr">
         <is>
-          <t>F01S Invoices insurer shares</t>
+          <t>F01S Invoice shares</t>
         </is>
       </c>
       <c r="B252" s="23" t="inlineStr">
@@ -15912,7 +15912,7 @@
     <row r="253">
       <c r="A253" s="12" t="inlineStr">
         <is>
-          <t>F01S Invoices insurer shares</t>
+          <t>F01S Invoice shares</t>
         </is>
       </c>
       <c r="B253" s="22" t="inlineStr">
@@ -15930,7 +15930,7 @@
     <row r="254">
       <c r="A254" s="14" t="inlineStr">
         <is>
-          <t>F01S Invoices insurer shares</t>
+          <t>F01S Invoice shares</t>
         </is>
       </c>
       <c r="B254" s="23" t="inlineStr">
@@ -15948,7 +15948,7 @@
     <row r="255">
       <c r="A255" s="12" t="inlineStr">
         <is>
-          <t>F01C Invoices components and</t>
+          <t>F01C Invoice components</t>
         </is>
       </c>
       <c r="B255" s="22" t="inlineStr">
@@ -15966,7 +15966,7 @@
     <row r="256">
       <c r="A256" s="14" t="inlineStr">
         <is>
-          <t>F01C Invoices components and</t>
+          <t>F01C Invoice components</t>
         </is>
       </c>
       <c r="B256" s="23" t="inlineStr">
@@ -15984,7 +15984,7 @@
     <row r="257">
       <c r="A257" s="12" t="inlineStr">
         <is>
-          <t>F01C Invoices components and</t>
+          <t>F01C Invoice components</t>
         </is>
       </c>
       <c r="B257" s="22" t="inlineStr">
@@ -16002,7 +16002,7 @@
     <row r="258">
       <c r="A258" s="14" t="inlineStr">
         <is>
-          <t>F01C Invoices components and</t>
+          <t>F01C Invoice components</t>
         </is>
       </c>
       <c r="B258" s="23" t="inlineStr">
@@ -16024,7 +16024,7 @@
     <row r="259">
       <c r="A259" s="12" t="inlineStr">
         <is>
-          <t>F01C Invoices components and</t>
+          <t>F01C Invoice components</t>
         </is>
       </c>
       <c r="B259" s="22" t="inlineStr">
@@ -16042,7 +16042,7 @@
     <row r="260">
       <c r="A260" s="14" t="inlineStr">
         <is>
-          <t>F01C Invoices components and</t>
+          <t>F01C Invoice components</t>
         </is>
       </c>
       <c r="B260" s="23" t="inlineStr">
@@ -16064,7 +16064,7 @@
     <row r="261">
       <c r="A261" s="12" t="inlineStr">
         <is>
-          <t>F01C Invoices components and</t>
+          <t>F01C Invoice components</t>
         </is>
       </c>
       <c r="B261" s="22" t="inlineStr">
@@ -16082,7 +16082,7 @@
     <row r="262">
       <c r="A262" s="14" t="inlineStr">
         <is>
-          <t>F01C Invoices components and</t>
+          <t>F01C Invoice components</t>
         </is>
       </c>
       <c r="B262" s="23" t="inlineStr">
@@ -16100,7 +16100,7 @@
     <row r="263">
       <c r="A263" s="12" t="inlineStr">
         <is>
-          <t>F01C Invoices components and</t>
+          <t>F01C Invoice components</t>
         </is>
       </c>
       <c r="B263" s="22" t="inlineStr">
@@ -16118,7 +16118,7 @@
     <row r="264">
       <c r="A264" s="14" t="inlineStr">
         <is>
-          <t>F01C Invoices components and</t>
+          <t>F01C Invoice components</t>
         </is>
       </c>
       <c r="B264" s="23" t="inlineStr">
@@ -16136,7 +16136,7 @@
     <row r="265">
       <c r="A265" s="12" t="inlineStr">
         <is>
-          <t>F01C Invoices components and</t>
+          <t>F01C Invoice components</t>
         </is>
       </c>
       <c r="B265" s="22" t="inlineStr">
@@ -16154,7 +16154,7 @@
     <row r="266">
       <c r="A266" s="14" t="inlineStr">
         <is>
-          <t>F01C Invoices components and</t>
+          <t>F01C Invoice components</t>
         </is>
       </c>
       <c r="B266" s="23" t="inlineStr">
@@ -16172,7 +16172,7 @@
     <row r="267">
       <c r="A267" s="12" t="inlineStr">
         <is>
-          <t>F02 Unapplied premium payments</t>
+          <t>F02 UPP</t>
         </is>
       </c>
       <c r="B267" s="22" t="inlineStr">
@@ -16190,7 +16190,7 @@
     <row r="268">
       <c r="A268" s="14" t="inlineStr">
         <is>
-          <t>F02 Unapplied premium payments</t>
+          <t>F02 UPP</t>
         </is>
       </c>
       <c r="B268" s="23" t="inlineStr">
@@ -16208,7 +16208,7 @@
     <row r="269">
       <c r="A269" s="12" t="inlineStr">
         <is>
-          <t>F02 Unapplied premium payments</t>
+          <t>F02 UPP</t>
         </is>
       </c>
       <c r="B269" s="22" t="inlineStr">
@@ -16226,7 +16226,7 @@
     <row r="270">
       <c r="A270" s="14" t="inlineStr">
         <is>
-          <t>F02 Unapplied premium payments</t>
+          <t>F02 UPP</t>
         </is>
       </c>
       <c r="B270" s="23" t="inlineStr">
@@ -16248,7 +16248,7 @@
     <row r="271">
       <c r="A271" s="12" t="inlineStr">
         <is>
-          <t>F02 Unapplied premium payments</t>
+          <t>F02 UPP</t>
         </is>
       </c>
       <c r="B271" s="22" t="inlineStr">
@@ -16266,7 +16266,7 @@
     <row r="272">
       <c r="A272" s="14" t="inlineStr">
         <is>
-          <t>F02 Unapplied premium payments</t>
+          <t>F02 UPP</t>
         </is>
       </c>
       <c r="B272" s="23" t="inlineStr">
@@ -16288,7 +16288,7 @@
     <row r="273">
       <c r="A273" s="12" t="inlineStr">
         <is>
-          <t>F02 Unapplied premium payments</t>
+          <t>F02 UPP</t>
         </is>
       </c>
       <c r="B273" s="22" t="inlineStr">
@@ -16306,7 +16306,7 @@
     <row r="274">
       <c r="A274" s="14" t="inlineStr">
         <is>
-          <t>F02 Unapplied premium payments</t>
+          <t>F02 UPP</t>
         </is>
       </c>
       <c r="B274" s="23" t="inlineStr">
@@ -16324,7 +16324,7 @@
     <row r="275">
       <c r="A275" s="12" t="inlineStr">
         <is>
-          <t>F02 Unapplied premium payments</t>
+          <t>F02 UPP</t>
         </is>
       </c>
       <c r="B275" s="22" t="inlineStr">
@@ -16342,7 +16342,7 @@
     <row r="276">
       <c r="A276" s="14" t="inlineStr">
         <is>
-          <t>F02 Unapplied premium payments</t>
+          <t>F02 UPP</t>
         </is>
       </c>
       <c r="B276" s="23" t="inlineStr">
@@ -16360,7 +16360,7 @@
     <row r="277">
       <c r="A277" s="12" t="inlineStr">
         <is>
-          <t>F02 Unapplied premium payments</t>
+          <t>F02 UPP</t>
         </is>
       </c>
       <c r="B277" s="22" t="inlineStr">
@@ -16378,7 +16378,7 @@
     <row r="278">
       <c r="A278" s="14" t="inlineStr">
         <is>
-          <t>F02 Unapplied premium payments</t>
+          <t>F02 UPP</t>
         </is>
       </c>
       <c r="B278" s="23" t="inlineStr">
@@ -16844,7 +16844,7 @@
     <row r="303">
       <c r="A303" s="12" t="inlineStr">
         <is>
-          <t>F06 PDCs, check pick-ups and</t>
+          <t>F06 PDCs pick-ups refunds</t>
         </is>
       </c>
       <c r="B303" s="22" t="inlineStr">
@@ -16862,7 +16862,7 @@
     <row r="304">
       <c r="A304" s="14" t="inlineStr">
         <is>
-          <t>F06 PDCs, check pick-ups and</t>
+          <t>F06 PDCs pick-ups refunds</t>
         </is>
       </c>
       <c r="B304" s="23" t="inlineStr">
@@ -16880,7 +16880,7 @@
     <row r="305">
       <c r="A305" s="12" t="inlineStr">
         <is>
-          <t>F06 PDCs, check pick-ups and</t>
+          <t>F06 PDCs pick-ups refunds</t>
         </is>
       </c>
       <c r="B305" s="22" t="inlineStr">
@@ -16898,7 +16898,7 @@
     <row r="306">
       <c r="A306" s="14" t="inlineStr">
         <is>
-          <t>F06 PDCs, check pick-ups and</t>
+          <t>F06 PDCs pick-ups refunds</t>
         </is>
       </c>
       <c r="B306" s="23" t="inlineStr">
@@ -16920,7 +16920,7 @@
     <row r="307">
       <c r="A307" s="12" t="inlineStr">
         <is>
-          <t>F06 PDCs, check pick-ups and</t>
+          <t>F06 PDCs pick-ups refunds</t>
         </is>
       </c>
       <c r="B307" s="22" t="inlineStr">
@@ -16938,7 +16938,7 @@
     <row r="308">
       <c r="A308" s="14" t="inlineStr">
         <is>
-          <t>F06 PDCs, check pick-ups and</t>
+          <t>F06 PDCs pick-ups refunds</t>
         </is>
       </c>
       <c r="B308" s="23" t="inlineStr">
@@ -16960,7 +16960,7 @@
     <row r="309">
       <c r="A309" s="12" t="inlineStr">
         <is>
-          <t>F06 PDCs, check pick-ups and</t>
+          <t>F06 PDCs pick-ups refunds</t>
         </is>
       </c>
       <c r="B309" s="22" t="inlineStr">
@@ -16978,7 +16978,7 @@
     <row r="310">
       <c r="A310" s="14" t="inlineStr">
         <is>
-          <t>F06 PDCs, check pick-ups and</t>
+          <t>F06 PDCs pick-ups refunds</t>
         </is>
       </c>
       <c r="B310" s="23" t="inlineStr">
@@ -16996,7 +16996,7 @@
     <row r="311">
       <c r="A311" s="12" t="inlineStr">
         <is>
-          <t>F06 PDCs, check pick-ups and</t>
+          <t>F06 PDCs pick-ups refunds</t>
         </is>
       </c>
       <c r="B311" s="22" t="inlineStr">
@@ -17014,7 +17014,7 @@
     <row r="312">
       <c r="A312" s="14" t="inlineStr">
         <is>
-          <t>F06 PDCs, check pick-ups and</t>
+          <t>F06 PDCs pick-ups refunds</t>
         </is>
       </c>
       <c r="B312" s="23" t="inlineStr">
@@ -17032,7 +17032,7 @@
     <row r="313">
       <c r="A313" s="12" t="inlineStr">
         <is>
-          <t>F06 PDCs, check pick-ups and</t>
+          <t>F06 PDCs pick-ups refunds</t>
         </is>
       </c>
       <c r="B313" s="22" t="inlineStr">
@@ -17050,7 +17050,7 @@
     <row r="314">
       <c r="A314" s="14" t="inlineStr">
         <is>
-          <t>F06 PDCs, check pick-ups and</t>
+          <t>F06 PDCs pick-ups refunds</t>
         </is>
       </c>
       <c r="B314" s="23" t="inlineStr">
@@ -17068,7 +17068,7 @@
     <row r="315">
       <c r="A315" s="12" t="inlineStr">
         <is>
-          <t>G01 GL opening trial balance</t>
+          <t>G01 GL trial balance</t>
         </is>
       </c>
       <c r="B315" s="22" t="inlineStr">
@@ -17086,7 +17086,7 @@
     <row r="316">
       <c r="A316" s="14" t="inlineStr">
         <is>
-          <t>G01 GL opening trial balance</t>
+          <t>G01 GL trial balance</t>
         </is>
       </c>
       <c r="B316" s="23" t="inlineStr">
@@ -17104,7 +17104,7 @@
     <row r="317">
       <c r="A317" s="12" t="inlineStr">
         <is>
-          <t>G01 GL opening trial balance</t>
+          <t>G01 GL trial balance</t>
         </is>
       </c>
       <c r="B317" s="22" t="inlineStr">
@@ -17122,7 +17122,7 @@
     <row r="318">
       <c r="A318" s="14" t="inlineStr">
         <is>
-          <t>G01 GL opening trial balance</t>
+          <t>G01 GL trial balance</t>
         </is>
       </c>
       <c r="B318" s="23" t="inlineStr">
@@ -17144,7 +17144,7 @@
     <row r="319">
       <c r="A319" s="12" t="inlineStr">
         <is>
-          <t>G01 GL opening trial balance</t>
+          <t>G01 GL trial balance</t>
         </is>
       </c>
       <c r="B319" s="22" t="inlineStr">
@@ -17162,7 +17162,7 @@
     <row r="320">
       <c r="A320" s="14" t="inlineStr">
         <is>
-          <t>G01 GL opening trial balance</t>
+          <t>G01 GL trial balance</t>
         </is>
       </c>
       <c r="B320" s="23" t="inlineStr">
@@ -17184,7 +17184,7 @@
     <row r="321">
       <c r="A321" s="12" t="inlineStr">
         <is>
-          <t>G01 GL opening trial balance</t>
+          <t>G01 GL trial balance</t>
         </is>
       </c>
       <c r="B321" s="22" t="inlineStr">
@@ -17202,7 +17202,7 @@
     <row r="322">
       <c r="A322" s="14" t="inlineStr">
         <is>
-          <t>G01 GL opening trial balance</t>
+          <t>G01 GL trial balance</t>
         </is>
       </c>
       <c r="B322" s="23" t="inlineStr">
@@ -17220,7 +17220,7 @@
     <row r="323">
       <c r="A323" s="12" t="inlineStr">
         <is>
-          <t>G01 GL opening trial balance</t>
+          <t>G01 GL trial balance</t>
         </is>
       </c>
       <c r="B323" s="22" t="inlineStr">
@@ -17238,7 +17238,7 @@
     <row r="324">
       <c r="A324" s="14" t="inlineStr">
         <is>
-          <t>G01 GL opening trial balance</t>
+          <t>G01 GL trial balance</t>
         </is>
       </c>
       <c r="B324" s="23" t="inlineStr">
@@ -17256,7 +17256,7 @@
     <row r="325">
       <c r="A325" s="12" t="inlineStr">
         <is>
-          <t>G01 GL opening trial balance</t>
+          <t>G01 GL trial balance</t>
         </is>
       </c>
       <c r="B325" s="22" t="inlineStr">
@@ -17274,7 +17274,7 @@
     <row r="326">
       <c r="A326" s="14" t="inlineStr">
         <is>
-          <t>G01 GL opening trial balance</t>
+          <t>G01 GL trial balance</t>
         </is>
       </c>
       <c r="B326" s="23" t="inlineStr">
@@ -17292,7 +17292,7 @@
     <row r="327">
       <c r="A327" s="12" t="inlineStr">
         <is>
-          <t>H01 Archive records closed</t>
+          <t>H01 Archive records</t>
         </is>
       </c>
       <c r="B327" s="22" t="inlineStr">
@@ -17310,7 +17310,7 @@
     <row r="328">
       <c r="A328" s="14" t="inlineStr">
         <is>
-          <t>H01 Archive records closed</t>
+          <t>H01 Archive records</t>
         </is>
       </c>
       <c r="B328" s="23" t="inlineStr">
@@ -17328,7 +17328,7 @@
     <row r="329">
       <c r="A329" s="12" t="inlineStr">
         <is>
-          <t>H01 Archive records closed</t>
+          <t>H01 Archive records</t>
         </is>
       </c>
       <c r="B329" s="22" t="inlineStr">
@@ -17346,7 +17346,7 @@
     <row r="330">
       <c r="A330" s="14" t="inlineStr">
         <is>
-          <t>H01 Archive records closed</t>
+          <t>H01 Archive records</t>
         </is>
       </c>
       <c r="B330" s="23" t="inlineStr">
@@ -17368,7 +17368,7 @@
     <row r="331">
       <c r="A331" s="12" t="inlineStr">
         <is>
-          <t>H01 Archive records closed</t>
+          <t>H01 Archive records</t>
         </is>
       </c>
       <c r="B331" s="22" t="inlineStr">
@@ -17386,7 +17386,7 @@
     <row r="332">
       <c r="A332" s="14" t="inlineStr">
         <is>
-          <t>H01 Archive records closed</t>
+          <t>H01 Archive records</t>
         </is>
       </c>
       <c r="B332" s="23" t="inlineStr">
@@ -17408,7 +17408,7 @@
     <row r="333">
       <c r="A333" s="12" t="inlineStr">
         <is>
-          <t>H01 Archive records closed</t>
+          <t>H01 Archive records</t>
         </is>
       </c>
       <c r="B333" s="22" t="inlineStr">
@@ -17426,7 +17426,7 @@
     <row r="334">
       <c r="A334" s="14" t="inlineStr">
         <is>
-          <t>H01 Archive records closed</t>
+          <t>H01 Archive records</t>
         </is>
       </c>
       <c r="B334" s="23" t="inlineStr">
@@ -17444,7 +17444,7 @@
     <row r="335">
       <c r="A335" s="12" t="inlineStr">
         <is>
-          <t>H01 Archive records closed</t>
+          <t>H01 Archive records</t>
         </is>
       </c>
       <c r="B335" s="22" t="inlineStr">
@@ -17462,7 +17462,7 @@
     <row r="336">
       <c r="A336" s="14" t="inlineStr">
         <is>
-          <t>H01 Archive records closed</t>
+          <t>H01 Archive records</t>
         </is>
       </c>
       <c r="B336" s="23" t="inlineStr">
@@ -17480,7 +17480,7 @@
     <row r="337">
       <c r="A337" s="12" t="inlineStr">
         <is>
-          <t>H01 Archive records closed</t>
+          <t>H01 Archive records</t>
         </is>
       </c>
       <c r="B337" s="22" t="inlineStr">
@@ -17498,7 +17498,7 @@
     <row r="338">
       <c r="A338" s="14" t="inlineStr">
         <is>
-          <t>H01 Archive records closed</t>
+          <t>H01 Archive records</t>
         </is>
       </c>
       <c r="B338" s="23" t="inlineStr">
@@ -17516,7 +17516,7 @@
     <row r="339">
       <c r="A339" s="12" t="inlineStr">
         <is>
-          <t>H02 Archive documents index</t>
+          <t>H02 Archive documents</t>
         </is>
       </c>
       <c r="B339" s="22" t="inlineStr">
@@ -17534,7 +17534,7 @@
     <row r="340">
       <c r="A340" s="14" t="inlineStr">
         <is>
-          <t>H02 Archive documents index</t>
+          <t>H02 Archive documents</t>
         </is>
       </c>
       <c r="B340" s="23" t="inlineStr">
@@ -17552,7 +17552,7 @@
     <row r="341">
       <c r="A341" s="12" t="inlineStr">
         <is>
-          <t>H02 Archive documents index</t>
+          <t>H02 Archive documents</t>
         </is>
       </c>
       <c r="B341" s="22" t="inlineStr">
@@ -17570,7 +17570,7 @@
     <row r="342">
       <c r="A342" s="14" t="inlineStr">
         <is>
-          <t>H02 Archive documents index</t>
+          <t>H02 Archive documents</t>
         </is>
       </c>
       <c r="B342" s="23" t="inlineStr">
@@ -17592,7 +17592,7 @@
     <row r="343">
       <c r="A343" s="12" t="inlineStr">
         <is>
-          <t>H02 Archive documents index</t>
+          <t>H02 Archive documents</t>
         </is>
       </c>
       <c r="B343" s="22" t="inlineStr">
@@ -17610,7 +17610,7 @@
     <row r="344">
       <c r="A344" s="14" t="inlineStr">
         <is>
-          <t>H02 Archive documents index</t>
+          <t>H02 Archive documents</t>
         </is>
       </c>
       <c r="B344" s="23" t="inlineStr">
@@ -17632,7 +17632,7 @@
     <row r="345">
       <c r="A345" s="12" t="inlineStr">
         <is>
-          <t>H02 Archive documents index</t>
+          <t>H02 Archive documents</t>
         </is>
       </c>
       <c r="B345" s="22" t="inlineStr">
@@ -17650,7 +17650,7 @@
     <row r="346">
       <c r="A346" s="14" t="inlineStr">
         <is>
-          <t>H02 Archive documents index</t>
+          <t>H02 Archive documents</t>
         </is>
       </c>
       <c r="B346" s="23" t="inlineStr">
@@ -17668,7 +17668,7 @@
     <row r="347">
       <c r="A347" s="12" t="inlineStr">
         <is>
-          <t>H02 Archive documents index</t>
+          <t>H02 Archive documents</t>
         </is>
       </c>
       <c r="B347" s="22" t="inlineStr">
@@ -17686,7 +17686,7 @@
     <row r="348">
       <c r="A348" s="14" t="inlineStr">
         <is>
-          <t>H02 Archive documents index</t>
+          <t>H02 Archive documents</t>
         </is>
       </c>
       <c r="B348" s="23" t="inlineStr">
@@ -17704,7 +17704,7 @@
     <row r="349">
       <c r="A349" s="12" t="inlineStr">
         <is>
-          <t>H02 Archive documents index</t>
+          <t>H02 Archive documents</t>
         </is>
       </c>
       <c r="B349" s="22" t="inlineStr">
@@ -17722,7 +17722,7 @@
     <row r="350">
       <c r="A350" s="14" t="inlineStr">
         <is>
-          <t>H02 Archive documents index</t>
+          <t>H02 Archive documents</t>
         </is>
       </c>
       <c r="B350" s="23" t="inlineStr">
@@ -19107,7 +19107,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="21" t="inlineStr">
         <is>
-          <t>P01S Policy insurer shares</t>
+          <t>P01S Policy shares</t>
         </is>
       </c>
     </row>
@@ -19612,7 +19612,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="21" t="inlineStr">
         <is>
-          <t>P03 RMEL cohorts already</t>
+          <t>P03 RMEL cohorts</t>
         </is>
       </c>
     </row>
@@ -20476,7 +20476,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="21" t="inlineStr">
         <is>
-          <t>F01 Invoices header</t>
+          <t>F01 Invoice header</t>
         </is>
       </c>
     </row>
@@ -22898,7 +22898,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="21" t="inlineStr">
         <is>
-          <t>F01S Invoices insurer shares</t>
+          <t>F01S Invoice shares</t>
         </is>
       </c>
     </row>
@@ -23343,7 +23343,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="21" t="inlineStr">
         <is>
-          <t>F01C Invoices components and</t>
+          <t>F01C Invoice components</t>
         </is>
       </c>
     </row>
@@ -23968,7 +23968,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="21" t="inlineStr">
         <is>
-          <t>F02 Unapplied premium payments</t>
+          <t>F02 UPP</t>
         </is>
       </c>
     </row>
@@ -26983,7 +26983,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="21" t="inlineStr">
         <is>
-          <t>F06 PDCs, check pick-ups and</t>
+          <t>F06 PDCs pick-ups refunds</t>
         </is>
       </c>
     </row>
@@ -27968,7 +27968,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="21" t="inlineStr">
         <is>
-          <t>G01 GL opening trial balance</t>
+          <t>G01 GL trial balance</t>
         </is>
       </c>
     </row>
@@ -31907,7 +31907,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="21" t="inlineStr">
         <is>
-          <t>H01 Archive records closed</t>
+          <t>H01 Archive records</t>
         </is>
       </c>
     </row>
@@ -32952,7 +32952,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="21" t="inlineStr">
         <is>
-          <t>H02 Archive documents index</t>
+          <t>H02 Archive documents</t>
         </is>
       </c>
     </row>
@@ -46267,7 +46267,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="21" t="inlineStr">
         <is>
-          <t>R01 Lists of values and MIS</t>
+          <t>R01 LOV and MIS values</t>
         </is>
       </c>
     </row>
@@ -46892,7 +46892,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="21" t="inlineStr">
         <is>
-          <t>R02 Branches and invoicing</t>
+          <t>R02 Branches</t>
         </is>
       </c>
     </row>
@@ -47337,7 +47337,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="21" t="inlineStr">
         <is>
-          <t>R03 Sales organisation units</t>
+          <t>R03 Sales organisation</t>
         </is>
       </c>
     </row>

</xml_diff>